<commit_message>
Actualizacion 17-Oct: presentacion optimizada en mobile landscape, chat consultivo reparado, desaturacion y coherencia total de matrices e informes
</commit_message>
<xml_diff>
--- a/Anexo_E_Matrices_MVP_Marley_Coffee.xlsx
+++ b/Anexo_E_Matrices_MVP_Marley_Coffee.xlsx
@@ -1917,7 +1917,7 @@
       </c>
       <c r="B27" s="6" t="inlineStr">
         <is>
-          <t>Atención en chat y WhatsApp de principio a fin: intenciones, datos mínimos, estados, traspaso humano, integración propuesta, permisos, fallos y criterios de aceptación.</t>
+          <t>Chat consultivo y seguimiento comercial por correo. WhatsApp solo para postventa iniciada por cliente: estados, traspaso, permisos y criterios de aceptación.</t>
         </is>
       </c>
     </row>
@@ -6111,7 +6111,7 @@
       </c>
       <c r="C35" s="10" t="inlineStr">
         <is>
-          <t>3 datos + permiso (nombre, correo y WhatsApp con +56 9 escrito); la comuna pasa al paso 2; con ellos se recupera a quien abandona</t>
+          <t>Nombre y correo + permiso para guardar el avance; teléfono opcional. La comuna pasa al paso 2; recuperación por correo</t>
         </is>
       </c>
       <c r="D35" s="10" t="inlineStr">
@@ -7138,7 +7138,7 @@
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
-          <t>Si el abandono en C03 es alto, pedir solo correo o WhatsApp al principio y el resto al aceptar.</t>
+          <t>Si el abandono en C03 es alto, pedir solo correo al principio y el resto al solicitar la propuesta.</t>
         </is>
       </c>
       <c r="H17" s="6" t="inlineStr">
@@ -7538,7 +7538,7 @@
       </c>
       <c r="C27" s="10" t="inlineStr">
         <is>
-          <t>A/B de canal destacado (chat vs llamada) en el piloto.</t>
+          <t>A/B de ayuda en chat y claridad del seguimiento por correo en el piloto.</t>
         </is>
       </c>
       <c r="D27" s="10" t="inlineStr">
@@ -8211,7 +8211,7 @@
       </c>
       <c r="B36" s="6" t="inlineStr">
         <is>
-          <t>El cliente elige chat, llamada o correo, pero los tres llegan a la misma conversación de su ejecutiva.</t>
+          <t>El chat asesora y conserva el contexto; la ejecutiva responde por correo con el resumen del mismo caso.</t>
         </is>
       </c>
     </row>
@@ -10723,7 +10723,7 @@
     <row r="15" ht="62" customHeight="1">
       <c r="A15" s="7" t="inlineStr">
         <is>
-          <t>Correo, WhatsApp, chat y teléfono</t>
+          <t>Chat consultivo, correo comercial y WhatsApp postventa entrante</t>
         </is>
       </c>
       <c r="B15" s="14" t="inlineStr">
@@ -10738,7 +10738,7 @@
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>W1/W4 mediante Connectif u orquestación; WhatsApp mediante plataforma oficial; Message Center no prueba nutrición comercial</t>
+          <t>W1/W4 por correo mediante Connectif u orquestación. WhatsApp solo postventa entrante; Message Center no prueba nutrición comercial</t>
         </is>
       </c>
       <c r="E15" s="14" t="inlineStr">
@@ -10874,7 +10874,7 @@
       </c>
       <c r="D21" s="10" t="inlineStr">
         <is>
-          <t>Correo, WhatsApp, chat y teléfono</t>
+          <t>Chat consultivo, correo comercial y WhatsApp postventa entrante</t>
         </is>
       </c>
       <c r="E21" s="10" t="inlineStr">
@@ -10906,7 +10906,7 @@
       </c>
       <c r="D22" s="10" t="inlineStr">
         <is>
-          <t>Correo, WhatsApp, chat y teléfono</t>
+          <t>Chat consultivo, correo comercial y WhatsApp postventa entrante</t>
         </is>
       </c>
       <c r="E22" s="10" t="inlineStr">
@@ -11194,7 +11194,7 @@
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>Correo, WhatsApp, chat y teléfono</t>
+          <t>Chat consultivo, correo comercial y WhatsApp postventa entrante</t>
         </is>
       </c>
       <c r="E31" s="10" t="inlineStr">
@@ -11226,7 +11226,7 @@
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>Correo, WhatsApp, chat y teléfono</t>
+          <t>Chat consultivo, correo comercial y WhatsApp postventa entrante</t>
         </is>
       </c>
       <c r="E32" s="10" t="inlineStr">
@@ -11995,7 +11995,7 @@
       </c>
       <c r="F57" s="10" t="inlineStr">
         <is>
-          <t>Correo, WhatsApp, chat y teléfono, VTEX IO (tienda actual), CRM Marley Coffee Empresas (propuesto)</t>
+          <t>Chat consultivo, correo comercial y WhatsApp postventa entrante, VTEX IO (tienda actual), CRM Marley Coffee Empresas (propuesto)</t>
         </is>
       </c>
       <c r="G57" s="6" t="inlineStr">
@@ -12416,7 +12416,7 @@
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>Formulario al principio (nombre, correo y WhatsApp con +56 9 escrito, y permiso); correo con el N.º de seguimiento; si abandona, aviso a las 24 h y audiencia de remarketing</t>
+          <t>Formulario al principio (nombre y correo, teléfono opcional y permiso); correo con N.º de seguimiento; si abandona, correo a las 24 h y remarketing autorizado</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
@@ -12426,7 +12426,7 @@
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>Sitio, correo y WhatsApp</t>
+          <t>Sitio y correo</t>
         </is>
       </c>
       <c r="H7" s="10" t="inlineStr">
@@ -12530,7 +12530,7 @@
       </c>
       <c r="E9" s="10" t="inlineStr">
         <is>
-          <t>Aceptar en un toque; chat con bot y espera visible; llamada con ficha que el cliente ve; la ejecutiva envía la propuesta que sugirió el agente</t>
+          <t>Revisar el resumen y solicitar propuesta por correo; el chat resuelve dudas y la ejecutiva confirma condiciones por correo</t>
         </is>
       </c>
       <c r="F9" s="10" t="inlineStr">
@@ -12540,7 +12540,7 @@
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>Portal, WhatsApp, teléfono y correo</t>
+          <t>Chat web y correo comercial</t>
         </is>
       </c>
       <c r="H9" s="10" t="inlineStr">
@@ -13018,7 +13018,7 @@
       </c>
       <c r="C29" s="10" t="inlineStr">
         <is>
-          <t>En el canal que elige la persona: chat con asistente y ejecutiva, llamada en vivo con ficha, correo o WhatsApp; la ejecutiva ve lo que cotizó y la propuesta que le sugiere el agente.</t>
+          <t>El chat web resuelve dudas y prepara el resumen. La ejecutiva recibe lo cotizado y responde por correo con las condiciones revisadas.</t>
         </is>
       </c>
       <c r="D29" s="6" t="inlineStr">
@@ -13040,7 +13040,7 @@
       </c>
       <c r="C30" s="10" t="inlineStr">
         <is>
-          <t>Audiencias con los datos que dejó al principio (correo y WhatsApp con permiso) y de quienes dejaron el diagnóstico a medias (Google y Meta), con la pieza de su negocio; se pausa cuando ya habló con una persona (W6).</t>
+          <t>Audiencias autorizadas de quienes dejaron el diagnóstico a medias (Google y Meta); recuperación por correo. Se pausa con atención humana activa (W6); sin WhatsApp comercial.</t>
         </is>
       </c>
       <c r="D30" s="6" t="inlineStr">
@@ -13651,7 +13651,7 @@
       </c>
       <c r="C13" s="10" t="inlineStr">
         <is>
-          <t>Elige canal de contacto</t>
+          <t>Confirma correo de contacto</t>
         </is>
       </c>
       <c r="D13" s="11" t="n">
@@ -13659,7 +13659,7 @@
       </c>
       <c r="E13" s="10" t="inlineStr">
         <is>
-          <t>Chat, llamada o correo.</t>
+          <t>Correo para seguimiento comercial.</t>
         </is>
       </c>
       <c r="F13" s="11" t="n">
@@ -15370,7 +15370,7 @@
       </c>
       <c r="C6" s="10" t="inlineStr">
         <is>
-          <t>Deja tu nombre y tu WhatsApp para que una ejecutiva de tu zona confirme tu propuesta de café para empresas.</t>
+          <t>Deja tu nombre y correo para que una ejecutiva de tu zona revise tu propuesta de café para empresas.</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -16160,7 +16160,7 @@
       </c>
       <c r="B45" s="10" t="inlineStr">
         <is>
-          <t>Sí. Te atiende la ejecutiva de tu zona por chat, llamada o correo, y ve tu diagnóstico para que no repitas nada.</t>
+          <t>Sí. El chat te orienta y la ejecutiva de tu zona responde por correo con tu diagnóstico para que no repitas nada.</t>
         </is>
       </c>
     </row>
@@ -17141,7 +17141,7 @@
     <row r="2" ht="16" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Propuesta de integración para el piloto; el prototipo demuestra el recorrido y no envía mensajes reales. El cliente conserva su contexto al pasar del sitio a WhatsApp y de la IA a una persona.</t>
+          <t>Propuesta de integración para el piloto; no envía mensajes reales. El chat conserva el contexto y la ejecutiva responde por correo. WhatsApp solo atiende postventa iniciada por el cliente.</t>
         </is>
       </c>
     </row>
@@ -17520,7 +17520,7 @@
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>Caso registrado, canal elegido y disponibilidad por confirmar; alternativa de correo</t>
+          <t>Caso registrado y respuesta comercial por correo; disponibilidad por confirmar</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
@@ -17643,7 +17643,7 @@
       </c>
       <c r="B22" s="10" t="inlineStr">
         <is>
-          <t>WhatsApp Business Platform mediante Cloud API; cuenta, número, proveedor y presupuesto por definir con Marley Coffee. Chat web y WhatsApp alimentan una bandeja CRM común.</t>
+          <t>Correo para seguimiento comercial y chat web consultivo. WhatsApp Business Platform solo para postventa iniciada por el cliente; cuenta, proveedor y presupuesto por definir. El CRM conserva contexto y responsable.</t>
         </is>
       </c>
       <c r="C22" s="6" t="inlineStr">
@@ -17779,7 +17779,7 @@
       </c>
       <c r="B30" s="10" t="inlineStr">
         <is>
-          <t>Para contactar por WhatsApp se requiere número o usuario entregado y permiso para mensajes posteriores. Registrar finalidad, origen, fecha y retiro; respetar bajas. Distinguir seguimiento de servicio y ofertas, sin casillas premarcadas.</t>
+          <t>El cliente inicia WhatsApp para postventa. Registrar finalidad, origen y retiro; una consulta de servicio no autoriza publicidad. El MVP no inicia mensajes ni campañas por este canal. Seguimiento comercial por correo autorizado.</t>
         </is>
       </c>
       <c r="C30" s="6" t="inlineStr">
@@ -17796,7 +17796,7 @@
       </c>
       <c r="B31" s="10" t="inlineStr">
         <is>
-          <t>La ventana de atención de 24 horas se abre y reinicia con cada mensaje del usuario. Para iniciar conversación y para escribir fuera de esa ventana se necesita plantilla aprobada; sin ella, no enviar. No asumir permiso de marketing por una consulta de servicio.</t>
+          <t>Atender solo la postventa que inicia el cliente dentro de las condiciones vigentes del canal. El MVP no inicia ni reabre conversaciones de WhatsApp con plantillas. Si no puede continuar, registrar el caso y ofrecer seguimiento por correo.</t>
         </is>
       </c>
       <c r="C31" s="6" t="inlineStr">
@@ -19250,7 +19250,7 @@
       </c>
       <c r="C32" s="6" t="inlineStr">
         <is>
-          <t>Chat web, correo y WhatsApp con su permiso. Pedido: Message Center. Nutrición: Connectif u orquestador; persona toma la atención.</t>
+          <t>Chat web consultivo y correo comercial. WhatsApp: postventa iniciada por cliente. Pedido: Message Center. Nutrición por correo autorizado.</t>
         </is>
       </c>
     </row>
@@ -22289,7 +22289,7 @@
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>Contactos que aceptan o eligen chat, llamada, correo o WhatsApp / propuestas vistas × 100</t>
+          <t>Contactos que solicitan revisión o propuesta por correo / propuestas vistas × 100</t>
         </is>
       </c>
       <c r="E8" s="10" t="inlineStr">
@@ -24340,7 +24340,7 @@
       </c>
       <c r="E7" s="10" t="inlineStr">
         <is>
-          <t>Acepta su propuesta o elige chat, llamada o correo (C05 → C06; si no dejó sus datos, C03)</t>
+          <t>Solicita revisión de su propuesta por correo (C05 → C06; si faltan datos, C03)</t>
         </is>
       </c>
       <c r="F7" s="10" t="inlineStr">
@@ -24355,12 +24355,12 @@
       </c>
       <c r="H7" s="10" t="inlineStr">
         <is>
-          <t>Chat / teléfono / correo / WhatsApp</t>
+          <t>Chat consultivo y correo comercial</t>
         </is>
       </c>
       <c r="I7" s="10" t="inlineStr">
         <is>
-          <t>Acepta: «¡Listo!» con quién, por dónde y cuándo; la ejecutiva confirma precio y fecha. Chat: bot de bienvenida y espera visible. Llamada: cola o agenda. Correo: acuse</t>
+          <t>Solicitud registrada con folio, resumen y correo. La ejecutiva revisa condiciones y responde por correo; no confirma contrato ni instalación</t>
         </is>
       </c>
       <c r="J7" s="10" t="inlineStr">
@@ -24407,7 +24407,7 @@
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
-          <t>Sin actividad ni ejecutiva asignada; permiso por finalidad; WhatsApp solo con plantilla aprobada cuando corresponda</t>
+          <t>Sin actividad ni atención humana activa; permiso por finalidad; recuperación solo por correo</t>
         </is>
       </c>
       <c r="G8" s="10" t="inlineStr">
@@ -24417,7 +24417,7 @@
       </c>
       <c r="H8" s="10" t="inlineStr">
         <is>
-          <t>Canal elegido + remarketing con permiso</t>
+          <t>Correo + remarketing con permiso</t>
         </is>
       </c>
       <c r="I8" s="10" t="inlineStr">
@@ -24479,7 +24479,7 @@
       </c>
       <c r="H9" s="10" t="inlineStr">
         <is>
-          <t>Su canal elegido</t>
+          <t>Correo</t>
         </is>
       </c>
       <c r="I9" s="10" t="inlineStr">
@@ -24526,7 +24526,7 @@
       </c>
       <c r="E10" s="10" t="inlineStr">
         <is>
-          <t>La ejecutiva responde o llama</t>
+          <t>La ejecutiva responde por correo</t>
         </is>
       </c>
       <c r="F10" s="10" t="inlineStr">
@@ -24603,7 +24603,7 @@
       </c>
       <c r="H11" s="10" t="inlineStr">
         <is>
-          <t>Portal / WhatsApp con permiso</t>
+          <t>Portal y correo; WhatsApp solo entrante</t>
         </is>
       </c>
       <c r="I11" s="10" t="inlineStr">
@@ -24727,7 +24727,7 @@
       </c>
       <c r="H13" s="10" t="inlineStr">
         <is>
-          <t>Portal / chat / WhatsApp con permiso</t>
+          <t>Portal/chat; WhatsApp postventa entrante</t>
         </is>
       </c>
       <c r="I13" s="10" t="inlineStr">
@@ -25924,7 +25924,7 @@
       </c>
       <c r="F25" s="10" t="inlineStr">
         <is>
-          <t>Chat, correo, llamada o WhatsApp con una ficha y responsable; propuesta base/ampliada.</t>
+          <t>Chat consultivo y correo con una ficha y responsable; propuesta base/ampliada.</t>
         </is>
       </c>
       <c r="G25" s="10" t="inlineStr">
@@ -25981,7 +25981,7 @@
       </c>
       <c r="E26" s="10" t="inlineStr">
         <is>
-          <t>Usar frecuencia de compra para preparar último pedido; cliente revisa cantidades y confirma; Logística valida ruta. Ofrecer WhatsApp con permiso, manteniendo todo en la ficha.</t>
+          <t>Preparar el último pedido según frecuencia; avisar por portal o correo. El cliente revisa y confirma; Logística valida ruta. WhatsApp solo si el cliente inicia postventa.</t>
         </is>
       </c>
       <c r="F26" s="10" t="inlineStr">
@@ -26048,7 +26048,7 @@
       </c>
       <c r="F27" s="10" t="inlineStr">
         <is>
-          <t>Portal/chat/WhatsApp → ticket único → estado y confirmación.</t>
+          <t>Portal/chat/WhatsApp entrante → ticket único → estado y confirmación.</t>
         </is>
       </c>
       <c r="G27" s="10" t="inlineStr">

</xml_diff>

<commit_message>
Actualiza recorrido productos y comodato y sincroniza entrega Marley
</commit_message>
<xml_diff>
--- a/Anexo_E_Matrices_MVP_Marley_Coffee.xlsx
+++ b/Anexo_E_Matrices_MVP_Marley_Coffee.xlsx
@@ -1626,10 +1626,8 @@
       <c r="B1" s="2" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Versión 1.8 · 15-10-2026 (arriendo, compra directa y atención continua) · citado desde el informe EP3 (secciones 1.1 a 1.7 y anexos).</t>
-        </is>
+      <c r="A2" s="3" t="str">
+        <v>Versión1.9 ·19-10-2026 · Modelo confirmado: comodato y compra mensual de insumos. Recorrido: Productos C10 → Máquinas C11 → Contacto C03 → Diagnóstico C04. El test15oct corresponde a la versión anterior; no valida estas mejoras.</v>
       </c>
     </row>
     <row r="3"/>
@@ -8300,15 +8298,11 @@
       </c>
     </row>
     <row r="44">
-      <c r="A44" s="5" t="inlineStr">
-        <is>
-          <t>Arriendo / compra directa</t>
-        </is>
-      </c>
-      <c r="B44" s="6" t="inlineStr">
-        <is>
-          <t>Arriendo: cuota mensual por la máquina, aparte del café. Compra directa: pago único por el equipo, aparte del café y los servicios. Montos académicos a validar; la ejecutiva confirma precio y condiciones.</t>
-        </is>
+      <c r="A44" s="5" t="str">
+        <v>Comodato y abastecimiento</v>
+      </c>
+      <c r="B44" s="6" t="str">
+        <v>Préstamo del equipo con compra mensual de insumos. La carga base se paga antes de instalar. Referencia bajo/medio flujo:1.491.220CLP netos; no es mensualidad ni precio de la máquina. Mínimo mensual y modelos pendientes de confirmación.</v>
       </c>
     </row>
     <row r="45">
@@ -12357,10 +12351,8 @@
           <t>Por tipo de negocio</t>
         </is>
       </c>
-      <c r="E6" s="10" t="inlineStr">
-        <is>
-          <t>Hero con video al scroll, pestañas por negocio y escenas de casos (C02, C08)</t>
-        </is>
+      <c r="E6" s="10" t="str">
+        <v>Home con valor, proceso y productos (C02); catálogo cotizador (C10) → máquinas y comodato (C11) → contacto y diagnóstico. Casos como apoyo (C08).</v>
       </c>
       <c r="F6" s="10" t="inlineStr">
         <is>
@@ -12372,10 +12364,8 @@
           <t>Sitio Empresas</t>
         </is>
       </c>
-      <c r="H6" s="10" t="inlineStr">
-        <is>
-          <t>«Ver mi solución» (+10)</t>
-        </is>
+      <c r="H6" s="10" t="str">
+        <v>Exploración C10 → C11; sin puntos por artículos, cantidades ni permiso implícito. Iniciar cotización conserva el evento existente, sin duplicarlo.</v>
       </c>
       <c r="I6" s="10" t="inlineStr">
         <is>
@@ -12387,10 +12377,8 @@
           <t>K01, K03</t>
         </is>
       </c>
-      <c r="K6" s="6" t="inlineStr">
-        <is>
-          <t>+10 → 10</t>
-        </is>
+      <c r="K6" s="6" t="str">
+        <v>Evento de cotización existente +10 una sola vez; explorar/agregar productos no suma puntos adicionales.</v>
       </c>
     </row>
     <row r="7">
@@ -12471,10 +12459,8 @@
           <t>Negocio × zona × banda de puntaje</t>
         </is>
       </c>
-      <c r="E8" s="10" t="inlineStr">
-        <is>
-          <t>Diagnóstico de 3 pasos y propuesta al instante con máquina, café al mes y precio mensual; extras recomendados por negocio</t>
-        </is>
+      <c r="E8" s="10" t="str">
+        <v>Diagnóstico de3capas; propuesta con equipo en comodato, selección de productos y consumo orientativo. Carga inicial y reposición por cotizar separadas; complementos opcionales.</v>
       </c>
       <c r="F8" s="10" t="inlineStr">
         <is>
@@ -12862,10 +12848,8 @@
           <t>SEO desde el día cero</t>
         </is>
       </c>
-      <c r="C22" s="10" t="inlineStr">
-        <is>
-          <t>Palabras clave definidas por buyer persona (gerente de A&amp;B de hotel, dueño de restaurante o cafetería, productor de eventos): «café para empresas», «máquina de café para hotel», «arriendo máquina de café», «coffee break para empresas». Una página por intención con H1 y H2 que responden la búsqueda.</t>
-        </is>
+      <c r="C22" s="10" t="str">
+        <v>Palabras clave definidas por buyer persona (gerente de A&amp;B de hotel, dueño de restaurante o cafetería, productor de eventos): «café para empresas», «máquina de café para hotel», «máquina de café en comodato», «coffee break para empresas». Una página por intención con H1 y H2 que responden la búsqueda.</v>
       </c>
       <c r="D22" s="6" t="inlineStr">
         <is>
@@ -14054,10 +14038,8 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Máquinas, café y servicios: rangos SUPUESTOS y calculadora de costo mensual</t>
-        </is>
+      <c r="A1" s="1" t="str">
+        <v>Comodato: carga inicial confirmada y consumo orientativo</v>
       </c>
       <c r="B1" s="2" t="n"/>
       <c r="C1" s="2" t="n"/>
@@ -14071,10 +14053,8 @@
       <c r="K1" s="2" t="n"/>
     </row>
     <row r="2" ht="16" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>SUPUESTOS ACADÉMICOS pedidos por el autor (12-10-2026), a validar con Marley Coffee. Solo la referencia pública (bolsas de 227 g) es un dato real. Montos en CLP sin IVA.</t>
-        </is>
+      <c r="A2" s="3" t="str">
+        <v>Actualización19oct2026: correo y presupuesto del ejecutivo aportados por Carlos Vargas. No existe oferta de compra/arriendo de máquina. Los cuatro tipos del sitio son referencias; el correo menciona tres modelos sin identificar. No hay tarifa mensual ni mínimo confirmados.</v>
       </c>
     </row>
     <row r="3"/>
@@ -14114,25 +14094,17 @@
           <t>Personal</t>
         </is>
       </c>
-      <c r="H4" s="4" t="inlineStr">
-        <is>
-          <t>Compra directa mín (pago único)</t>
-        </is>
-      </c>
-      <c r="I4" s="4" t="inlineStr">
-        <is>
-          <t>Compra directa máx (pago único)</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Arriendo mín / mes</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>Arriendo máx / mes</t>
-        </is>
+      <c r="H4" s="4" t="str">
+        <v>Régimen del equipo</v>
+      </c>
+      <c r="I4" s="4" t="str">
+        <v>Disponibilidad</v>
+      </c>
+      <c r="J4" s="4" t="str">
+        <v>Tarifa del equipo</v>
+      </c>
+      <c r="K4" s="4" t="str">
+        <v>Validación</v>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
@@ -14171,17 +14143,17 @@
           <t>Con barista (capacitación a confirmar)</t>
         </is>
       </c>
-      <c r="H5" s="60" t="n">
-        <v>2900000</v>
-      </c>
-      <c r="I5" s="60" t="n">
-        <v>4500000</v>
-      </c>
-      <c r="J5" s="60" t="n">
-        <v>140000</v>
-      </c>
-      <c r="K5" s="62" t="n">
-        <v>220000</v>
+      <c r="H5" s="60" t="str">
+        <v>Comodato</v>
+      </c>
+      <c r="I5" s="60" t="str">
+        <v>Modelo por confirmar</v>
+      </c>
+      <c r="J5" s="60" t="str">
+        <v>No se ofrece venta/arriendo</v>
+      </c>
+      <c r="K5" s="62" t="str">
+        <v>Ejecutiva valida</v>
       </c>
     </row>
     <row r="6" ht="36" customHeight="1">
@@ -14220,17 +14192,17 @@
           <t>Autoservicio de un toque</t>
         </is>
       </c>
-      <c r="H6" s="60" t="n">
-        <v>1900000</v>
-      </c>
-      <c r="I6" s="60" t="n">
-        <v>3200000</v>
-      </c>
-      <c r="J6" s="60" t="n">
-        <v>65000</v>
-      </c>
-      <c r="K6" s="62" t="n">
-        <v>110000</v>
+      <c r="H6" s="60" t="str">
+        <v>Comodato</v>
+      </c>
+      <c r="I6" s="60" t="str">
+        <v>Modelo por confirmar</v>
+      </c>
+      <c r="J6" s="60" t="str">
+        <v>No se ofrece venta/arriendo</v>
+      </c>
+      <c r="K6" s="62" t="str">
+        <v>Ejecutiva valida</v>
       </c>
     </row>
     <row r="7" ht="36" customHeight="1">
@@ -14269,21 +14241,17 @@
           <t>Sin barista</t>
         </is>
       </c>
-      <c r="H7" s="60" t="inlineStr">
-        <is>
-          <t>A cotizar</t>
-        </is>
-      </c>
-      <c r="I7" s="60" t="inlineStr">
-        <is>
-          <t>A cotizar</t>
-        </is>
-      </c>
-      <c r="J7" s="60" t="n">
-        <v>95000</v>
-      </c>
-      <c r="K7" s="62" t="n">
-        <v>150000</v>
+      <c r="H7" s="60" t="str">
+        <v>Comodato</v>
+      </c>
+      <c r="I7" s="60" t="str">
+        <v>Modelo por confirmar</v>
+      </c>
+      <c r="J7" s="60" t="str">
+        <v>No se ofrece venta/arriendo</v>
+      </c>
+      <c r="K7" s="62" t="str">
+        <v>Ejecutiva valida</v>
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
@@ -14322,17 +14290,17 @@
           <t>Sin barista</t>
         </is>
       </c>
-      <c r="H8" s="63" t="n">
-        <v>690000</v>
-      </c>
-      <c r="I8" s="63" t="n">
-        <v>1200000</v>
-      </c>
-      <c r="J8" s="63" t="n">
-        <v>45000</v>
-      </c>
-      <c r="K8" s="64" t="n">
-        <v>80000</v>
+      <c r="H8" s="63" t="str">
+        <v>Comodato</v>
+      </c>
+      <c r="I8" s="63" t="str">
+        <v>Modelo por confirmar</v>
+      </c>
+      <c r="J8" s="63" t="str">
+        <v>No se ofrece venta/arriendo</v>
+      </c>
+      <c r="K8" s="64" t="str">
+        <v>Ejecutiva valida</v>
       </c>
     </row>
     <row r="9" ht="23" customHeight="1"/>
@@ -14389,22 +14357,20 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="C11" s="60" t="n">
-        <v>19900</v>
-      </c>
-      <c r="D11" s="60" t="n">
-        <v>25900</v>
+      <c r="C11" s="60" t="str">
+        <v>Por cotizar</v>
+      </c>
+      <c r="D11" s="60" t="str">
+        <v>Por cotizar</v>
       </c>
       <c r="E11" s="11" t="n">
         <v>110</v>
       </c>
-      <c r="F11" s="61">
-        <f>C11/E11</f>
-        <v/>
-      </c>
-      <c r="G11" s="61">
-        <f>D11/E11</f>
-        <v/>
+      <c r="F11" s="61" t="str">
+        <v>Por cotizar</v>
+      </c>
+      <c r="G11" s="61" t="str">
+        <v>Por cotizar</v>
       </c>
       <c r="H11" s="6" t="inlineStr">
         <is>
@@ -14423,22 +14389,20 @@
           <t>pod</t>
         </is>
       </c>
-      <c r="C12" s="60" t="n">
-        <v>290</v>
-      </c>
-      <c r="D12" s="60" t="n">
-        <v>390</v>
+      <c r="C12" s="60" t="str">
+        <v>Por cotizar</v>
+      </c>
+      <c r="D12" s="60" t="str">
+        <v>Por cotizar</v>
       </c>
       <c r="E12" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="61">
-        <f>C12/E12</f>
-        <v/>
-      </c>
-      <c r="G12" s="61">
-        <f>D12/E12</f>
-        <v/>
+      <c r="F12" s="61" t="str">
+        <v>Por cotizar</v>
+      </c>
+      <c r="G12" s="61" t="str">
+        <v>Por cotizar</v>
       </c>
       <c r="H12" s="6" t="inlineStr">
         <is>
@@ -14457,22 +14421,20 @@
           <t>kg</t>
         </is>
       </c>
-      <c r="C13" s="63" t="n">
-        <v>9900</v>
-      </c>
-      <c r="D13" s="63" t="n">
-        <v>13900</v>
+      <c r="C13" s="63" t="str">
+        <v>Por cotizar</v>
+      </c>
+      <c r="D13" s="63" t="str">
+        <v>Por cotizar</v>
       </c>
       <c r="E13" s="15" t="n">
         <v>60</v>
       </c>
-      <c r="F13" s="65">
-        <f>C13/E13</f>
-        <v/>
-      </c>
-      <c r="G13" s="65">
-        <f>D13/E13</f>
-        <v/>
+      <c r="F13" s="65" t="str">
+        <v>Por cotizar</v>
+      </c>
+      <c r="G13" s="65" t="str">
+        <v>Por cotizar</v>
       </c>
       <c r="H13" s="8" t="inlineStr">
         <is>
@@ -14524,11 +14486,11 @@
           <t>Barra Marley Coffee con barista, tazas y material de marca para tu evento.</t>
         </is>
       </c>
-      <c r="C16" s="60" t="n">
-        <v>450000</v>
-      </c>
-      <c r="D16" s="60" t="n">
-        <v>780000</v>
+      <c r="C16" s="60" t="str">
+        <v>Por cotizar</v>
+      </c>
+      <c r="D16" s="60" t="str">
+        <v>Por cotizar</v>
       </c>
       <c r="E16" s="10" t="inlineStr">
         <is>
@@ -14552,11 +14514,11 @@
           <t>Coffee break con mantel, tazas y café Marley Coffee para reuniones y lanzamientos.</t>
         </is>
       </c>
-      <c r="C17" s="60" t="n">
-        <v>5900</v>
-      </c>
-      <c r="D17" s="60" t="n">
-        <v>8900</v>
+      <c r="C17" s="60" t="str">
+        <v>Por cotizar</v>
+      </c>
+      <c r="D17" s="60" t="str">
+        <v>Por cotizar</v>
       </c>
       <c r="E17" s="10" t="inlineStr">
         <is>
@@ -14580,11 +14542,11 @@
           <t>Un módulo Marley Coffee con barista en tu local, hotel o centro comercial por una temporada.</t>
         </is>
       </c>
-      <c r="C18" s="60" t="n">
-        <v>380000</v>
-      </c>
-      <c r="D18" s="60" t="n">
-        <v>650000</v>
+      <c r="C18" s="60" t="str">
+        <v>Por cotizar</v>
+      </c>
+      <c r="D18" s="60" t="str">
+        <v>Por cotizar</v>
       </c>
       <c r="E18" s="10" t="inlineStr">
         <is>
@@ -14608,11 +14570,11 @@
           <t>Frente de barra, piso modular, exhibidor de bolsas y carta con la marca.</t>
         </is>
       </c>
-      <c r="C19" s="60" t="n">
-        <v>150000</v>
-      </c>
-      <c r="D19" s="60" t="n">
-        <v>420000</v>
+      <c r="C19" s="60" t="str">
+        <v>Por cotizar</v>
+      </c>
+      <c r="D19" s="60" t="str">
+        <v>Por cotizar</v>
       </c>
       <c r="E19" s="10" t="inlineStr">
         <is>
@@ -14636,11 +14598,11 @@
           <t>Tu equipo aprende a preparar y cuidar la máquina con un barista de Marley Coffee.</t>
         </is>
       </c>
-      <c r="C20" s="60" t="n">
-        <v>90000</v>
-      </c>
-      <c r="D20" s="60" t="n">
-        <v>140000</v>
+      <c r="C20" s="60" t="str">
+        <v>Por cotizar</v>
+      </c>
+      <c r="D20" s="60" t="str">
+        <v>Por cotizar</v>
       </c>
       <c r="E20" s="10" t="inlineStr">
         <is>
@@ -14664,11 +14626,11 @@
           <t>Taza mug negra y travel mug Marley Coffee para tu servicio.</t>
         </is>
       </c>
-      <c r="C21" s="60" t="n">
-        <v>6500</v>
-      </c>
-      <c r="D21" s="60" t="n">
-        <v>8900</v>
+      <c r="C21" s="60" t="str">
+        <v>Por cotizar</v>
+      </c>
+      <c r="D21" s="60" t="str">
+        <v>Por cotizar</v>
       </c>
       <c r="E21" s="10" t="inlineStr">
         <is>
@@ -14774,10 +14736,8 @@
     </row>
     <row r="27" ht="23" customHeight="1"/>
     <row r="28" ht="36" customHeight="1">
-      <c r="A28" s="50" t="inlineStr">
-        <is>
-          <t>Calculadora de costo mensual (cambia las celdas amarillas)</t>
-        </is>
+      <c r="A28" s="50" t="str">
+        <v>Consumo orientativo y pago antes de instalar (magnitudes separadas)</v>
       </c>
     </row>
     <row r="29" ht="23" customHeight="1">
@@ -14818,10 +14778,8 @@
           <t>Modalidad</t>
         </is>
       </c>
-      <c r="B32" s="11" t="inlineStr">
-        <is>
-          <t>arriendo</t>
-        </is>
+      <c r="B32" s="11" t="str">
+        <v>comodato</v>
       </c>
     </row>
     <row r="33" ht="23" customHeight="1">
@@ -14847,122 +14805,91 @@
       </c>
     </row>
     <row r="35" ht="23" customHeight="1">
-      <c r="A35" s="10" t="inlineStr">
-        <is>
-          <t>Insumo al mes mín</t>
-        </is>
-      </c>
-      <c r="B35" s="61">
-        <f>B34*IF(B29="pods",C12,C11)</f>
-        <v/>
+      <c r="A35" s="10" t="str">
+        <v>Reposición mensual · precio mínimo</v>
+      </c>
+      <c r="B35" s="61" t="str">
+        <v>Por confirmar con el equipo</v>
       </c>
     </row>
     <row r="36" ht="23" customHeight="1">
-      <c r="A36" s="10" t="inlineStr">
-        <is>
-          <t>Insumo al mes máx</t>
-        </is>
-      </c>
-      <c r="B36" s="61">
-        <f>B34*IF(B29="pods",D12,D11)</f>
-        <v/>
+      <c r="A36" s="10" t="str">
+        <v>Reposición mensual · precio máximo</v>
+      </c>
+      <c r="B36" s="61" t="str">
+        <v>Por confirmar con el equipo</v>
       </c>
     </row>
     <row r="37" ht="36" customHeight="1">
-      <c r="A37" s="10" t="inlineStr">
-        <is>
-          <t>Cuota de la máquina mín (arriendo)</t>
-        </is>
-      </c>
-      <c r="B37" s="61">
-        <f>IF(B32="arriendo",INDEX($J$5:$J$8,MATCH(B29,$A$5:$A$8,0)),0)</f>
-        <v/>
+      <c r="A37" s="10" t="str">
+        <v>Carga base de insumos · neto</v>
+      </c>
+      <c r="B37" s="61" t="n">
+        <v>1331220</v>
       </c>
     </row>
     <row r="38" ht="36" customHeight="1">
-      <c r="A38" s="10" t="inlineStr">
-        <is>
-          <t>Cuota de la máquina máx (arriendo)</t>
-        </is>
-      </c>
-      <c r="B38" s="61">
-        <f>IF(B32="arriendo",INDEX($K$5:$K$8,MATCH(B29,$A$5:$A$8,0)),0)</f>
-        <v/>
+      <c r="A38" s="10" t="str">
+        <v>Kit de instalación · neto</v>
+      </c>
+      <c r="B38" s="61" t="n">
+        <v>100000</v>
       </c>
     </row>
     <row r="39" ht="36" customHeight="1">
-      <c r="A39" s="10" t="inlineStr">
-        <is>
-          <t>Total mensual mín (café + arriendo si aplica)</t>
-        </is>
-      </c>
-      <c r="B39" s="61">
-        <f>IF(ISNUMBER(B37),B35+B37,"A cotizar")</f>
-        <v/>
+      <c r="A39" s="10" t="str">
+        <v>Filtro · neto</v>
+      </c>
+      <c r="B39" s="61" t="n">
+        <v>60000</v>
       </c>
     </row>
     <row r="40" ht="36" customHeight="1">
-      <c r="A40" s="10" t="inlineStr">
-        <is>
-          <t>Total mensual máx (café + arriendo si aplica)</t>
-        </is>
-      </c>
-      <c r="B40" s="61">
-        <f>IF(ISNUMBER(B38),B36+B38,"A cotizar")</f>
-        <v/>
+      <c r="A40" s="10" t="str">
+        <v>Total antes de instalar · neto</v>
+      </c>
+      <c r="B40" s="61" t="n">
+        <f>SUM(B37:B39)</f>
+        <v>1491220</v>
       </c>
     </row>
     <row r="41" ht="23" customHeight="1">
-      <c r="A41" s="10" t="inlineStr">
-        <is>
-          <t>Pago único (compra directa) mín</t>
-        </is>
-      </c>
-      <c r="B41" s="61">
-        <f>IF(B32="compra",INDEX($H$5:$H$8,MATCH(B29,$A$5:$A$8,0)),0)</f>
-        <v/>
+      <c r="A41" s="10" t="str">
+        <v>Mínimo mensual de compra</v>
+      </c>
+      <c r="B41" s="61" t="str">
+        <v>Por confirmar con el equipo</v>
       </c>
     </row>
     <row r="42" ht="23" customHeight="1">
-      <c r="A42" s="10" t="inlineStr">
-        <is>
-          <t>Pago único (compra directa) máx</t>
-        </is>
-      </c>
-      <c r="B42" s="61">
-        <f>IF(B32="compra",INDEX($I$5:$I$8,MATCH(B29,$A$5:$A$8,0)),0)</f>
-        <v/>
+      <c r="A42" s="10" t="str">
+        <v>Modelo disponible</v>
+      </c>
+      <c r="B42" s="61" t="str">
+        <v>Por confirmar con el equipo</v>
       </c>
     </row>
     <row r="43" ht="36" customHeight="1">
-      <c r="A43" s="10" t="inlineStr">
-        <is>
-          <t>Costo por taza mín (mensual ÷ tazas al mes)</t>
-        </is>
-      </c>
-      <c r="B43" s="61">
-        <f>IF(AND(ISNUMBER(B39),B30*B31&gt;0),B39/(B30*B31),"A cotizar")</f>
-        <v/>
+      <c r="A43" s="10" t="str">
+        <v>Costo por taza mínimo</v>
+      </c>
+      <c r="B43" s="61" t="str">
+        <v>Por confirmar con el equipo</v>
       </c>
     </row>
     <row r="44" ht="36" customHeight="1">
-      <c r="A44" s="10" t="inlineStr">
-        <is>
-          <t>Costo por taza máx (mensual ÷ tazas al mes)</t>
-        </is>
-      </c>
-      <c r="B44" s="61">
-        <f>IF(AND(ISNUMBER(B40),B30*B31&gt;0),B40/(B30*B31),"A cotizar")</f>
-        <v/>
+      <c r="A44" s="10" t="str">
+        <v>Costo por taza máximo</v>
+      </c>
+      <c r="B44" s="61" t="str">
+        <v>Por confirmar con el equipo</v>
       </c>
     </row>
     <row r="45" ht="23" customHeight="1"/>
     <row r="46" ht="23" customHeight="1"/>
     <row r="47" ht="36" customHeight="1">
-      <c r="A47" s="50" t="inlineStr">
-        <is>
-          <t>Dos formas de adquirir la máquina</t>
-        </is>
+      <c r="A47" s="50" t="str">
+        <v>Modelo comercial confirmado</v>
       </c>
     </row>
     <row r="48" ht="30" customHeight="1">
@@ -14988,81 +14915,54 @@
       </c>
     </row>
     <row r="49" ht="62" customHeight="1">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>Arriendo</t>
-        </is>
-      </c>
-      <c r="B49" s="10" t="inlineStr">
-        <is>
-          <t>Disponible en el diseño del MVP</t>
-        </is>
-      </c>
-      <c r="C49" s="10" t="inlineStr">
-        <is>
-          <t>Alcance acordado con el autor, 15-10-2026; rangos académicos a validar con Marley Coffee</t>
-        </is>
-      </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>Cuota mensual por el equipo, café y extras separados; la ejecutiva confirma precio y condiciones.</t>
-        </is>
+      <c r="A49" s="5" t="str">
+        <v>Comodato</v>
+      </c>
+      <c r="B49" s="10" t="str">
+        <v>Confirmado por correo del ejecutivo</v>
+      </c>
+      <c r="C49" s="10" t="str">
+        <v>19-10-2026 · correo y presupuesto aportados por Carlos Vargas</v>
+      </c>
+      <c r="D49" s="6" t="str">
+        <v>Máquina prestada con compra mensual de insumos; carga base se paga antes de instalar.</v>
       </c>
     </row>
     <row r="50" ht="75" customHeight="1">
-      <c r="A50" s="5" t="inlineStr">
-        <is>
-          <t>Compra directa</t>
-        </is>
-      </c>
-      <c r="B50" s="10" t="inlineStr">
-        <is>
-          <t>Disponible en el diseño del MVP</t>
-        </is>
-      </c>
-      <c r="C50" s="10" t="inlineStr">
-        <is>
-          <t>Alcance acordado con el autor, 15-10-2026; no se presenta como oferta oficial vigente</t>
-        </is>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>Pago único por máquina, aparte del café; si no existe rango sustentado: A cotizar. Precio y condiciones sujetos a confirmación.</t>
-        </is>
+      <c r="A50" s="5" t="str">
+        <v>Abastecimiento mensual</v>
+      </c>
+      <c r="B50" s="10" t="str">
+        <v>Precio, mínimo y formatos por confirmar</v>
+      </c>
+      <c r="C50" s="10" t="str">
+        <v>No fueron detallados en la comunicación recibida</v>
+      </c>
+      <c r="D50" s="6" t="str">
+        <v>Productos elegidos y cantidades son una solicitud para cotizar, no una compra ni un pedido confirmado.</v>
       </c>
     </row>
     <row r="51" ht="88" customHeight="1">
-      <c r="A51" s="7" t="inlineStr">
-        <is>
-          <t>Lectura de la calculadora</t>
-        </is>
-      </c>
-      <c r="B51" s="14" t="inlineStr">
-        <is>
-          <t>Montos CLP sin IVA; sin extras ni instalación</t>
-        </is>
-      </c>
-      <c r="C51" s="14" t="inlineStr">
-        <is>
-          <t>Supuestos académicos, no tarifa comercial</t>
-        </is>
-      </c>
-      <c r="D51" s="8" t="inlineStr">
-        <is>
-          <t>El total mensual suma café y arriendo cuando aplica; el pago único de compra directa se muestra aparte. Con 250 tazas/día × 26 días: 6.500 tazas/mes; grano a 110 tazas/kg.</t>
-        </is>
+      <c r="A51" s="7" t="str">
+        <v>Cómo leer las cifras</v>
+      </c>
+      <c r="B51" s="14" t="str">
+        <v>Montos netos CLP; referencia bajo/medio flujo</v>
+      </c>
+      <c r="C51" s="14" t="str">
+        <v>Carga inicial:1.331.220 +100.000 +60.000 =1.491.220</v>
+      </c>
+      <c r="D51" s="8" t="str">
+        <v>La carga base no se repite automáticamente cada mes ni se recalcula desde el carrito. El consumo de250tazas/día ×26días /110tazas/kg =59,09kg/mes es supuesto operativo, no mínimo contractual.</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:K2"/>
   </mergeCells>
-  <dataValidations count="2">
+  <dataValidations count="1">
     <dataValidation sqref="B29" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>=$A$5:$A$8</formula1>
-    </dataValidation>
-    <dataValidation sqref="B32" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" errorTitle="Elige una modalidad" error="Solo arriendo o compra directa." type="list" errorStyle="stop">
-      <formula1>"arriendo,compra"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15346,10 +15246,8 @@
           <t>Café para empresas, hoteles y restaurantes | Marley Coffee Empresas</t>
         </is>
       </c>
-      <c r="C5" s="10" t="inlineStr">
-        <is>
-          <t>Máquinas de café en arriendo o compra directa, café orgánico y servicios para eventos. Recomendación en 1 minuto y ejecutiva de tu zona.</t>
-        </is>
+      <c r="C5" s="10" t="str">
+        <v>Máquinas de café en comodato con compra mensual de insumos, café orgánico y servicios para eventos. Recomendación en 1 minuto y ejecutiva de tu zona.</v>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
@@ -15601,10 +15499,8 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
-        <is>
-          <t>arriendo máquina de café</t>
-        </is>
+      <c r="A18" s="5" t="str">
+        <v>máquina de café en comodato</v>
       </c>
       <c r="B18" s="10" t="inlineStr">
         <is>
@@ -15616,10 +15512,8 @@
           <t>C07 cotizador</t>
         </is>
       </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>Arriendo mensual con café separado y compra directa de equipo</t>
-        </is>
+      <c r="D18" s="6" t="str">
+        <v>Condiciones de comodato y compra mensual de insumos, sin oferta de arriendo o venta de equipo.</v>
       </c>
     </row>
     <row r="19">
@@ -15788,15 +15682,11 @@
           <t>De una taza a todo tu local</t>
         </is>
       </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>Máquinas de café en arriendo o compra directa</t>
-        </is>
-      </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>arriendo / compra máquina de café</t>
-        </is>
+      <c r="D27" s="10" t="str">
+        <v>Máquinas de café en comodato con compra mensual de insumos</v>
+      </c>
+      <c r="E27" s="6" t="str">
+        <v>máquina en comodato y abastecimiento de café</v>
       </c>
     </row>
     <row r="28">
@@ -15869,10 +15759,8 @@
           <t>Elige por cómo sirves, no por catálogo</t>
         </is>
       </c>
-      <c r="D30" s="10" t="inlineStr">
-        <is>
-          <t>Máquinas de café para empresas: arriendo o compra directa</t>
-        </is>
+      <c r="D30" s="10" t="str">
+        <v>Máquinas de café para empresas: comodato con compra mensual de insumos</v>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
@@ -16110,10 +15998,8 @@
           <t>¿Puedo arrendar o comprar la máquina?</t>
         </is>
       </c>
-      <c r="B41" s="10" t="inlineStr">
-        <is>
-          <t>Puedes elegir arriendo mensual o compra directa. El consumo de café se calcula aparte y la ejecutiva confirma precio, instalación y condiciones. Los valores mostrados son supuestos académicos; donde falta precio de compra se indica A cotizar.</t>
-        </is>
+      <c r="B41" s="10" t="str">
+        <v>La máquina se presta en comodato con compra mensual de insumos. La carga inicial de referencia para bajo/medio flujo es1.491.220CLP netos, antes de instalar. Modelo, formatos, compatibilidad, mínimo mensual y precios de reposición se confirman con el equipo; no se vende ni arrienda la máquina.</v>
       </c>
     </row>
     <row r="42">
@@ -17194,10 +17080,8 @@
           <t>Explorar y comparar</t>
         </is>
       </c>
-      <c r="B5" s="10" t="inlineStr">
-        <is>
-          <t>Elegir máquina; comparar arriendo y compra directa</t>
-        </is>
+      <c r="B5" s="10" t="str">
+        <v>Explorar productos y máquinas; entender comodato, carga inicial y reposición por cotizar.</v>
       </c>
       <c r="C5" s="10" t="inlineStr">
         <is>
@@ -18096,10 +17980,8 @@
           <t>Modalidades</t>
         </is>
       </c>
-      <c r="B48" s="10" t="inlineStr">
-        <is>
-          <t>Arriendo mensual y compra directa. Montos de demostración académica; precio, stock, cobertura y condiciones los confirma la ejecutiva.</t>
-        </is>
+      <c r="B48" s="10" t="str">
+        <v>Comodato con compra mensual de insumos. Montos de demostración académica; precio, stock, cobertura y condiciones los confirma la ejecutiva.</v>
       </c>
     </row>
   </sheetData>
@@ -24124,10 +24006,8 @@
       <c r="L1" s="2" t="n"/>
     </row>
     <row r="2" ht="26" customHeight="1">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>Adaptados del Anexo B (W1–W9, fuentes M1, M2, P1 y P2) al recorrido v6.1 (15-10: los datos básicos se piden al principio, antes del diagnóstico; si la persona abandona, W4 la recupera). Regla: un canal a la vez y solo con permiso; la toma humana pausa las secuencias.</t>
-        </is>
+      <c r="A2" s="3" t="str">
+        <v>Recorrido vigente19oct: C02 → C10 Productos → C11 Máquinas/condiciones → C03 Contacto → C04 Diagnóstico → C05 Propuesta → C06 Folio. W1 solo con correo y permiso; la cesta no crea consentimiento ni puntaje. Edición posterior exige nueva revisión; W4/W5 por correo y WhatsApp solo en postventa entrante.</v>
       </c>
     </row>
     <row r="3"/>
@@ -24214,10 +24094,8 @@
           <t>Identificación</t>
         </is>
       </c>
-      <c r="E5" s="10" t="inlineStr">
-        <is>
-          <t>Deja sus datos con permiso al empezar (C03, antes del diagnóstico)</t>
-        </is>
+      <c r="E5" s="10" t="str">
+        <v>Tras explorar productos (C10) y máquinas (C11), deja datos con permiso (C03, antes del diagnóstico)</v>
       </c>
       <c r="F5" s="10" t="inlineStr">
         <is>
@@ -24249,10 +24127,8 @@
           <t>K02</t>
         </is>
       </c>
-      <c r="L5" s="6" t="inlineStr">
-        <is>
-          <t>Aviso de correo; R01</t>
-        </is>
+      <c r="L5" s="6" t="str">
+        <v>C10/C11 preceden a C03; correo local y R01. Productos/cantidades y preferencia conservados hasta R02/R08.</v>
       </c>
     </row>
     <row r="6" ht="75" customHeight="1">
@@ -25421,10 +25297,8 @@
           <t>Administración de hoteles, restaurantes, cafeterías y eventos</t>
         </is>
       </c>
-      <c r="E17" s="10" t="inlineStr">
-        <is>
-          <t>Crear /empresas y páginas útiles por negocio; enlazar desde Empresas, catálogo pertinente y guías. Explicar arriendo y compra directa con respuestas propias de cada operación.</t>
-        </is>
+      <c r="E17" s="10" t="str">
+        <v>Crear /empresas y páginas útiles por negocio; enlazar desde Empresas, catálogo pertinente y guías. Explicar comodato y abastecimiento mensual con respuestas propias de cada operación.</v>
       </c>
       <c r="F17" s="10" t="inlineStr">
         <is>
@@ -25545,10 +25419,8 @@
           <t>Quien compara proveedores o modalidades para su negocio</t>
         </is>
       </c>
-      <c r="E19" s="10" t="inlineStr">
-        <is>
-          <t>Separar grupos: arriendo de máquina, compra de máquina y café HORECA; anuncios y página de destino coherentes con cada búsqueda. Revisar términos y negativas de consumo doméstico, empleo, reparación ajena y búsquedas no atendibles; verificar contexto antes de excluir.</t>
-        </is>
+      <c r="E19" s="10" t="str">
+        <v>Separar intención de abastecimiento HORECA, equipos en comodato y café por negocio. Anuncio y destino explican el servicio real; excluir ofertas de venta/arriendo de equipos no disponibles. Medir términos y calidad de contactos, sin prometer posiciones ni rentabilidad.</v>
       </c>
       <c r="F19" s="10" t="inlineStr">
         <is>
@@ -26260,10 +26132,8 @@
           <t>/empresas/restaurantes (URL propuesta)</t>
         </is>
       </c>
-      <c r="E32" s="10" t="inlineStr">
-        <is>
-          <t>Contenido sobre servicio de sobremesa; comparar Pods sin barista y Bar con equipo; explicar arriendo y compra directa.</t>
-        </is>
+      <c r="E32" s="10" t="str">
+        <v>Contenido sobre servicio de sobremesa; comparar Pods sin barista y Bar con equipo; explicar comodato y abastecimiento mensual.</v>
       </c>
       <c r="F32" s="10" t="inlineStr">
         <is>
@@ -26386,25 +26256,17 @@
           <t>SEM · T03</t>
         </is>
       </c>
-      <c r="B35" s="10" t="inlineStr">
-        <is>
-          <t>Demanda de arriendo</t>
-        </is>
-      </c>
-      <c r="C35" s="10" t="inlineStr">
-        <is>
-          <t>Campaña Search Empresas / grupo Arriendo</t>
-        </is>
-      </c>
-      <c r="D35" s="10" t="inlineStr">
-        <is>
-          <t>/empresas/maquinas (URL propuesta; selección arriendo)</t>
-        </is>
-      </c>
-      <c r="E35" s="10" t="inlineStr">
-        <is>
-          <t>Anuncio ejemplo: «Café para tu negocio · Compara máquinas en arriendo». Términos por validar: arriendo máquina café empresa/hotel.</t>
-        </is>
+      <c r="B35" s="10" t="str">
+        <v>Demanda de comodato</v>
+      </c>
+      <c r="C35" s="10" t="str">
+        <v>Campaña Search Empresas / grupo Comodato</v>
+      </c>
+      <c r="D35" s="10" t="str">
+        <v>/empresas/maquinas (URL propuesta; condiciones de comodato)</v>
+      </c>
+      <c r="E35" s="10" t="str">
+        <v>Ejemplo propuesto: Café para tu negocio · equipo en comodato con compra mensual de insumos. Destino conecta catálogo y equipos antes de contacto. Términos por validar.</v>
       </c>
       <c r="F35" s="10" t="inlineStr">
         <is>
@@ -26433,25 +26295,17 @@
           <t>SEM · T03</t>
         </is>
       </c>
-      <c r="B36" s="10" t="inlineStr">
-        <is>
-          <t>Demanda de compra</t>
-        </is>
-      </c>
-      <c r="C36" s="10" t="inlineStr">
-        <is>
-          <t>Campaña Search Empresas / grupo Compra directa</t>
-        </is>
-      </c>
-      <c r="D36" s="10" t="inlineStr">
-        <is>
-          <t>/empresas/maquinas (URL propuesta; selección compra)</t>
-        </is>
-      </c>
-      <c r="E36" s="10" t="inlineStr">
-        <is>
-          <t>Anuncio ejemplo: «Máquina de café para tu negocio · Evalúa compra directa». Comparación con pago único y café aparte.</t>
-        </is>
+      <c r="B36" s="10" t="str">
+        <v>Demanda de abastecimiento</v>
+      </c>
+      <c r="C36" s="10" t="str">
+        <v>Campaña Search Empresas / grupo Insumos</v>
+      </c>
+      <c r="D36" s="10" t="str">
+        <v>/empresas/productos (URL propuesta; catálogo B2B)</v>
+      </c>
+      <c r="E36" s="10" t="str">
+        <v>Ejemplo propuesto: Café e insumos para tu negocio · arma tu abastecimiento. Precio profesional y formatos sujetos a validación; no usar precio público B2C como tarifa mayorista.</v>
       </c>
       <c r="F36" s="10" t="inlineStr">
         <is>

</xml_diff>